<commit_message>
Fix static tag in base template
</commit_message>
<xml_diff>
--- a/test data.xlsx
+++ b/test data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bbc6436f63d94ee7/Desktop/Attendance/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="8_{FC154A3E-B707-4AA5-A7C6-A2A064BA02FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3321BF24-A6E9-47FB-9163-32463C99D855}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="8_{FC154A3E-B707-4AA5-A7C6-A2A064BA02FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C33235A-B5F7-488E-B245-BFEDB5B075CF}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{6DE715AD-5EC9-4019-8D27-88DA0153E153}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
   <si>
     <t>Roll No</t>
   </si>
@@ -45,70 +45,64 @@
     <t>Registration No</t>
   </si>
   <si>
-    <t>Rona1ket</t>
-  </si>
-  <si>
-    <t>Rona2ket</t>
-  </si>
-  <si>
-    <t>Rona3ket</t>
-  </si>
-  <si>
-    <t>Rona4ket</t>
-  </si>
-  <si>
-    <t>Rona5ket</t>
-  </si>
-  <si>
-    <t>Rona11ket</t>
-  </si>
-  <si>
-    <t>Rona12ket</t>
-  </si>
-  <si>
-    <t>Rona13ket</t>
-  </si>
-  <si>
-    <t>Rona14ket</t>
-  </si>
-  <si>
-    <t>Rona15ket</t>
-  </si>
-  <si>
-    <t>Rona22ket</t>
-  </si>
-  <si>
-    <t>Rona23ket</t>
-  </si>
-  <si>
-    <t>Rona24ket</t>
-  </si>
-  <si>
-    <t>Rona25ket</t>
-  </si>
-  <si>
-    <t>Rona31ket</t>
-  </si>
-  <si>
-    <t>Rona32ket</t>
-  </si>
-  <si>
-    <t>Rona33ket</t>
-  </si>
-  <si>
-    <t>Rona34ket</t>
-  </si>
-  <si>
-    <t>Rona35ket</t>
-  </si>
-  <si>
-    <t>Rona41ket</t>
-  </si>
-  <si>
-    <t>Rona42ket</t>
-  </si>
-  <si>
-    <t>Rona43ket</t>
+    <t>Soca1ket</t>
+  </si>
+  <si>
+    <t>Soca2ket</t>
+  </si>
+  <si>
+    <t>Soca3ket</t>
+  </si>
+  <si>
+    <t>Soca4ket</t>
+  </si>
+  <si>
+    <t>Soca5ket</t>
+  </si>
+  <si>
+    <t>Soca131ket</t>
+  </si>
+  <si>
+    <t>Soca12ket</t>
+  </si>
+  <si>
+    <t>Soca13ket</t>
+  </si>
+  <si>
+    <t>Soca14ket</t>
+  </si>
+  <si>
+    <t>Soca15ket</t>
+  </si>
+  <si>
+    <t>Soca22ket</t>
+  </si>
+  <si>
+    <t>Soca23ket</t>
+  </si>
+  <si>
+    <t>Soca24ket</t>
+  </si>
+  <si>
+    <t>Soca25ket</t>
+  </si>
+  <si>
+    <t>Soca31ket</t>
+  </si>
+  <si>
+    <t>Soca32ket</t>
+  </si>
+  <si>
+    <t>Soca33ket</t>
+  </si>
+  <si>
+    <t>Soca34ket</t>
+  </si>
+  <si>
+    <t>Soca35ket</t>
+  </si>
+  <si>
+    <t>Soca41ket</t>
   </si>
 </sst>
 </file>
@@ -468,7 +462,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC43E5FE-B95E-4551-98E4-CABA6083B27E}">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -484,255 +478,233 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2">
-        <v>1101</v>
+        <v>13101</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
       </c>
       <c r="C2">
-        <v>55141</v>
+        <v>535141</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3">
-        <v>1102</v>
+        <v>13102</v>
       </c>
       <c r="B3" t="s">
         <v>4</v>
       </c>
       <c r="C3">
-        <v>55142</v>
+        <v>535142</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4">
-        <v>1103</v>
+        <v>13103</v>
       </c>
       <c r="B4" t="s">
         <v>5</v>
       </c>
       <c r="C4">
-        <v>55143</v>
+        <v>535143</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5">
-        <v>1104</v>
+        <v>13104</v>
       </c>
       <c r="B5" t="s">
         <v>6</v>
       </c>
       <c r="C5">
-        <v>55144</v>
+        <v>535144</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6">
-        <v>1105</v>
+        <v>13105</v>
       </c>
       <c r="B6" t="s">
         <v>7</v>
       </c>
       <c r="C6">
-        <v>55145</v>
+        <v>535145</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7">
-        <v>1106</v>
+        <v>13106</v>
       </c>
       <c r="B7" t="s">
         <v>8</v>
       </c>
       <c r="C7">
-        <v>55146</v>
+        <v>535146</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8">
-        <v>1107</v>
+        <v>13107</v>
       </c>
       <c r="B8" t="s">
         <v>9</v>
       </c>
       <c r="C8">
-        <v>55147</v>
+        <v>535147</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9">
-        <v>1108</v>
+        <v>13108</v>
       </c>
       <c r="B9" t="s">
         <v>10</v>
       </c>
       <c r="C9">
-        <v>55148</v>
+        <v>535148</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10">
-        <v>1109</v>
+        <v>13109</v>
       </c>
       <c r="B10" t="s">
         <v>11</v>
       </c>
       <c r="C10">
-        <v>55149</v>
+        <v>535149</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11">
-        <v>1110</v>
+        <v>13110</v>
       </c>
       <c r="B11" t="s">
         <v>12</v>
       </c>
       <c r="C11">
-        <v>55150</v>
+        <v>535150</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12">
-        <v>111</v>
+        <v>1311</v>
       </c>
       <c r="B12" t="s">
         <v>9</v>
       </c>
       <c r="C12">
-        <v>551551</v>
+        <v>53515351</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13">
-        <v>112</v>
+        <v>1312</v>
       </c>
       <c r="B13" t="s">
         <v>13</v>
       </c>
       <c r="C13">
-        <v>55152</v>
+        <v>535152</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14">
-        <v>113</v>
+        <v>1313</v>
       </c>
       <c r="B14" t="s">
         <v>14</v>
       </c>
       <c r="C14">
-        <v>55153</v>
+        <v>535153</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15">
-        <v>114</v>
+        <v>1314</v>
       </c>
       <c r="B15" t="s">
         <v>15</v>
       </c>
       <c r="C15">
-        <v>55154</v>
+        <v>535154</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16">
-        <v>115</v>
+        <v>1315</v>
       </c>
       <c r="B16" t="s">
         <v>16</v>
       </c>
       <c r="C16">
-        <v>55155</v>
+        <v>5351535</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17">
-        <v>116</v>
+        <v>1316</v>
       </c>
       <c r="B17" t="s">
         <v>17</v>
       </c>
       <c r="C17">
-        <v>55156</v>
+        <v>535156</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18">
-        <v>117</v>
+        <v>1317</v>
       </c>
       <c r="B18" t="s">
         <v>18</v>
       </c>
       <c r="C18">
-        <v>55157</v>
+        <v>535157</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19">
-        <v>118</v>
+        <v>1318</v>
       </c>
       <c r="B19" t="s">
         <v>19</v>
       </c>
       <c r="C19">
-        <v>55158</v>
+        <v>535158</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20">
-        <v>119</v>
+        <v>1319</v>
       </c>
       <c r="B20" t="s">
         <v>20</v>
       </c>
       <c r="C20">
-        <v>55159</v>
+        <v>535159</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21">
-        <v>120</v>
+        <v>1320</v>
       </c>
       <c r="B21" t="s">
         <v>21</v>
       </c>
       <c r="C21">
-        <v>55160</v>
+        <v>535160</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22">
-        <v>121</v>
+        <v>1321</v>
       </c>
       <c r="B22" t="s">
         <v>22</v>
       </c>
       <c r="C22">
-        <v>55161</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3">
-      <c r="A23">
-        <v>122</v>
-      </c>
-      <c r="B23" t="s">
-        <v>23</v>
-      </c>
-      <c r="C23">
-        <v>55162</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3">
-      <c r="A24">
-        <v>123</v>
-      </c>
-      <c r="B24" t="s">
-        <v>24</v>
-      </c>
-      <c r="C24">
-        <v>55163</v>
+        <v>535161</v>
       </c>
     </row>
   </sheetData>

</xml_diff>